<commit_message>
Phone: progress 1, log 1 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -2952,19 +2952,19 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-22</v>
       </c>
       <c r="N4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="str">
         <v>2.5</v>
       </c>
       <c r="P4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -2985,10 +2985,10 @@
         <v>0.12</v>
       </c>
       <c r="X4" t="str">
-        <v>9.74</v>
+        <v>9.79</v>
       </c>
       <c r="Y4" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-22</v>
       </c>
       <c r="Z4" t="str">
         <v/>
@@ -3058,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H234"/>
+  <dimension ref="A1:H235"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -9154,10 +9154,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B235" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C235" t="str">
+        <v>2026-09-22T11:50:42.936Z</v>
+      </c>
+      <c r="D235" t="str">
+        <v>again</v>
+      </c>
+      <c r="E235" t="str">
+        <v>18</v>
+      </c>
+      <c r="F235" t="str">
+        <v>0.12</v>
+      </c>
+      <c r="G235" t="str">
+        <v>9.79</v>
+      </c>
+      <c r="H235" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H234"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H235"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>